<commit_message>
scan: seg6 2026-06-23 01:13 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq7_2026-06-22.xlsx
+++ b/output/full_scan/batch_seq7_2026-06-22.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>71.83804001825058</v>
+        <v>71.83804001212292</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>42.51982205909755</v>
+        <v>42.51982208958855</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>2.862294443236175</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>2.601127507719445</v>
+        <v>2.601127508234589</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>63.53907619724571</v>
+        <v>63.53907618339679</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>22.8591232843241</v>
+        <v>22.85912322598512</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>2.040958598179007</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>7.167216444000445</v>
+        <v>7.1672164449277</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>65.8107894813123</v>
+        <v>65.81078944890146</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>25.55566872604825</v>
+        <v>25.55566868161306</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>1.421602804367013</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.5094384135345726</v>
+        <v>0.5094384136891186</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>69.09024072924271</v>
+        <v>69.09024069856281</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>33.4296425826101</v>
+        <v>33.42964256535509</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>2.319345784424896</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>1.072266112304484</v>
+        <v>1.07226611269597</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>62.52383794837784</v>
+        <v>62.52383787971241</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>27.93261515705605</v>
+        <v>27.93261520038898</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>1.633353219239842</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.4600424055000673</v>
+        <v>0.4600424059121848</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>68.33850695863271</v>
+        <v>68.33850694631599</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>26.91032928744684</v>
+        <v>26.910329254918</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>1.380767958988565</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>2.023318031902585</v>
+        <v>2.023318031985019</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>59.33549290599187</v>
+        <v>59.33549288444707</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>17.98445566704801</v>
+        <v>17.98445564082421</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>1.736693673720097</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>3.261973164074169</v>
+        <v>3.261973164795308</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>66.44782823390008</v>
+        <v>66.44782801088422</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>28.22758939479371</v>
+        <v>28.22758944763418</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>2.020486831555961</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.5157450982482603</v>
+        <v>0.5157450987634051</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>67.26172504275011</v>
+        <v>67.26172499187837</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>33.14913888083569</v>
+        <v>33.14913885997254</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>1.248347283904206</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.0024341283702224</v>
+        <v>0.0024341285968851</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>58.67740734772445</v>
+        <v>58.67740728475282</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>16.30240268404291</v>
+        <v>16.3024026070116</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>1.052144126389212</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.9648241480284314</v>
+        <v>0.9648241500889396</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>86.72513745991924</v>
+        <v>86.72513740865114</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>63.85568995130125</v>
+        <v>63.85568995147482</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>1.544734744213764</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>2.828445332810301</v>
+        <v>2.828445332707274</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>76.44948963361732</v>
+        <v>76.44948961661592</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>30.16663401027396</v>
+        <v>30.16663401026339</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>2.969853817875921</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>2.226142043172288</v>
+        <v>2.226142043316532</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>75.41572087347605</v>
+        <v>75.41572087394786</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>46.22877074754653</v>
+        <v>46.22877069810954</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>2.385124244880403</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>2.357274044753289</v>
+        <v>2.357274044876928</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>63.37881290379392</v>
+        <v>63.37881290745698</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>25.40389573081834</v>
+        <v>25.4038957724756</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>1.258908889109759</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>-3.669873189676444</v>
+        <v>-3.669873190088609</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>70.51705786031812</v>
+        <v>70.51705777650497</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>24.9891037263504</v>
+        <v>24.98910373902371</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>2.790809890551313</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.6799760688940338</v>
+        <v>0.6799760689558552</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,7 +1347,7 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>65.27891781870719</v>
+        <v>65.27891784958456</v>
       </c>
       <c r="I17" s="2" t="n">
         <v>13.60981439777852</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>1.600857355407189</v>
+        <v>1.600857355922366</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>61.64493178963191</v>
+        <v>61.64493178232065</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>23.41523210118356</v>
+        <v>23.41523202197185</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0.5156833425254695</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>-0.2010397750645274</v>
+        <v>-0.2010397750130108</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>61.58680573977691</v>
+        <v>61.58680572335353</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>23.57012891341498</v>
+        <v>23.57012877827464</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0.8806438698873151</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>-3.041480579120808</v>
+        <v>-3.041480577472221</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>78.12142297779705</v>
+        <v>78.12142297162598</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>45.7278848438592</v>
+        <v>45.72788485710802</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>0.5877561146265479</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>6.867348916847025</v>
+        <v>6.867348916826423</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>61.72335919616582</v>
+        <v>61.7233591243047</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>34.83885684042191</v>
+        <v>34.83885723303501</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>1.811182692842985</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>1.396184178961654</v>
+        <v>1.396184182567649</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>63.18390287886221</v>
+        <v>63.18390286761296</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>21.09442385744705</v>
+        <v>21.09442386231752</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>0.7105144700989028</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>8.922400540254163</v>
+        <v>8.922400540975366</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>67.04841650612642</v>
+        <v>67.04841649484959</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>13.70203792432854</v>
+        <v>13.70203792082034</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>1.144970098910921</v>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>58.05813342310773</v>
+        <v>58.05813344040367</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>31.25156125277458</v>
+        <v>31.25156120482127</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.6895794563734119</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.0242776624750526</v>
+        <v>0.0242776623308182</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>58.75978634692383</v>
+        <v>58.7597862893802</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>20.20039892112931</v>
+        <v>20.2003989332946</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>2.500312355246946</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>6.577953342178386</v>
+        <v>6.577953344857169</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>70.77725256544902</v>
+        <v>70.77725251933143</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>34.56597054188325</v>
+        <v>34.56597056532313</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>1.921618820419468</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>1.433139466282618</v>
+        <v>1.433139466437165</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>61.35745263790749</v>
+        <v>61.35745252596273</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>30.86742653583944</v>
+        <v>30.86742649617682</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0.5012741454082797</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.1104997714782645</v>
+        <v>0.1104997716843203</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>64.10400412668996</v>
+        <v>64.10400402475781</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>33.86795632243792</v>
+        <v>33.8679563138496</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>1.364925100856852</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.7757631603057127</v>
+        <v>0.7757631605117761</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>76.66809799973434</v>
+        <v>76.66809801302327</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>51.3885925174121</v>
+        <v>51.38859247907218</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>1.605069555625185</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>3.828075579400629</v>
+        <v>3.828075579153353</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>67.00952818409161</v>
+        <v>67.0095281305652</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>36.51869830322525</v>
+        <v>36.51869834787956</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>1.334496794784486</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>1.432607231534517</v>
+        <v>1.432607231287243</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>60.26981259048366</v>
+        <v>60.2698125745542</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>20.43165990857205</v>
+        <v>20.4316598078096</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>1.684927786226356</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>-0.4105333917065068</v>
+        <v>-0.4105333915416735</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>777.6684045833143</v>
+        <v>777.6684045833169</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>79.8</v>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>75.60909531076278</v>
+        <v>75.60909523836858</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>30.45101321935118</v>
+        <v>30.45101338576878</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.8195234080785511</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.6181293420083582</v>
+        <v>0.6181293425029104</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>67.38639719987046</v>
+        <v>67.38639717374176</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>34.37071735808468</v>
+        <v>34.37071737108052</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>2.472064333993977</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.6140599704155472</v>
+        <v>0.6140599705185767</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2251,7 +2251,7 @@
         <v>60.65759832128553</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>28.261929963627</v>
+        <v>28.26192999467911</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0.7723246604999969</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.3342219566000306</v>
+        <v>0.3342219563527542</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>58.21624301881637</v>
+        <v>58.2162429835492</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>24.29570352831795</v>
+        <v>24.29570341227562</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>1.557575651901278</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>-0.5103404321262226</v>
+        <v>-0.5103404317347118</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>67.58363344543409</v>
+        <v>67.58363344635309</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>45.69694267168143</v>
+        <v>45.69694269631884</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.5214001742173271</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>0.06405723469084811</v>
+        <v>0.0640572345981187</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2407,7 +2407,7 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>73.62156583529104</v>
+        <v>73.621565824464</v>
       </c>
       <c r="I37" s="2" t="n">
         <v>42.04139603425941</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.4099733589970291</v>
+        <v>0.4099733590382408</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>61.37942677517916</v>
+        <v>61.37942658259174</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>31.64296211765246</v>
+        <v>31.64296219595679</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>1.440607676157675</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.222358146024317</v>
+        <v>0.222358146343706</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>52.24837182471985</v>
+        <v>52.24837177713879</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>9.472178586115239</v>
+        <v>9.47217862033896</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>1.015936823541252</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>0.5036838192742374</v>
+        <v>0.5036838196863522</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>55.39142656172572</v>
+        <v>55.39142647540072</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>23.82078298282969</v>
+        <v>23.82078290153978</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.72442843775369</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>-1.346514544213179</v>
+        <v>-1.346514544316202</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>62.74579606069799</v>
+        <v>62.74579603174226</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>49.30024322429984</v>
+        <v>49.30024315735786</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.7094221588092477</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-0.3124169648606472</v>
+        <v>-0.3124169644897421</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2658,7 +2658,7 @@
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>692.3504879173499</v>
+        <v>692.3504879173501</v>
       </c>
       <c r="E42" s="2" t="n">
         <v>72.5</v>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>55.92901045329304</v>
+        <v>55.92900998580637</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>44.98928103021785</v>
+        <v>44.98928097014901</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.8148466688496909</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0.0192046976059688</v>
+        <v>0.0192046981829305</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>52.5967022042317</v>
+        <v>52.59670220703209</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>20.15571801574464</v>
+        <v>20.15571810879284</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>1.379634536928255</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-6.508109055626512</v>
+        <v>-6.508109055853229</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2764,7 +2764,7 @@
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>689.6243067464834</v>
+        <v>689.6243067464832</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>9460</v>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>53.39399747859505</v>
+        <v>53.39399747533329</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>20.61194074037965</v>
+        <v>20.61194066996485</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.7777632536177569</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>115.8502380753123</v>
+        <v>115.8502380757254</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>57.25952589072492</v>
+        <v>57.25952577975849</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>20.17789944774871</v>
+        <v>20.17789944007504</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.7808031480622462</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-0.1040100032832569</v>
+        <v>-0.1040100036953592</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>61.92488429781865</v>
+        <v>61.92488418575408</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>26.90267383455092</v>
+        <v>26.90267399174554</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.5274915518670342</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-1.179261779119429</v>
+        <v>-1.179261775822522</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>640.3478886488223</v>
+        <v>640.3478886488222</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>1205</v>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>54.66052400591636</v>
+        <v>54.66052393066374</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>13.32583661502721</v>
+        <v>13.32583652499959</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.8806751484776628</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>4.006688960209122</v>
+        <v>4.006688971748424</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>55.16867212374667</v>
+        <v>55.16867209368141</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>16.0609491722327</v>
+        <v>16.06094909175966</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>3.020106765995172</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.6575287620832073</v>
+        <v>0.6575287619801835</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>59.9377101515507</v>
+        <v>59.93771005874606</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>33.93993751089747</v>
+        <v>33.93993753271555</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>0.9356042563022812</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-1.084478074707896</v>
+        <v>-1.084478074192761</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>62.33847530010723</v>
+        <v>62.33847527310134</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>31.3151872680376</v>
+        <v>31.31518737532504</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>1.167266380030503</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-1.043630659827885</v>
+        <v>-1.043630659333338</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>52.83617412543013</v>
+        <v>52.83617402747232</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>31.37079515917764</v>
+        <v>31.37079526213276</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>1.813796421464137</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.2333746406024672</v>
+        <v>0.2333746400873178</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>51.23045956506296</v>
+        <v>51.23045954817567</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>17.3505407188313</v>
+        <v>17.35054063711223</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.5721717611502463</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>31.97559796664796</v>
+        <v>31.97559797076907</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3241,7 +3241,7 @@
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>596.9908006843475</v>
+        <v>596.9908006843474</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>54</v>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>54.5021759775878</v>
+        <v>54.50217591379585</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>12.77697921071769</v>
+        <v>12.77697913400967</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.7949757004807149</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.1156440862102377</v>
+        <v>0.1156440863441749</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>52.27566011374176</v>
+        <v>52.27566011458968</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>8.809622758206844</v>
+        <v>8.809622758206842</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>1.806814669013507</v>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>52.19599579828429</v>
+        <v>52.19599572456491</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>18.87793432346065</v>
+        <v>18.87793424735628</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.4689300272944461</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-0.603602211613519</v>
+        <v>-0.6036022113044335</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>52.92775678800818</v>
+        <v>52.9277566549896</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>15.40260868447633</v>
+        <v>15.40260868514711</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>1.243723469333888</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.0388116474699958</v>
+        <v>0.0388116475936309</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>56.68778939516305</v>
+        <v>56.68778934550759</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>16.19843960188613</v>
+        <v>16.19843955020303</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.8987760267500172</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-0.1275353532321946</v>
+        <v>-0.1275353530776535</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>59.55337968746401</v>
+        <v>59.55337966114536</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>24.23566309039644</v>
+        <v>24.235663105339</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>1.244596206946077</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.0596692697871837</v>
+        <v>0.0596692699211212</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>31.69502813815237</v>
+        <v>31.69502801993506</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>32.59319577751519</v>
+        <v>32.59319589058759</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>2.013053626871306</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.4112821516959535</v>
+        <v>0.4112821522523093</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>51.53517553567966</v>
+        <v>51.53517549981756</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>22.79029130644073</v>
+        <v>22.79029136931089</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>1.091842602001216</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.4569208077110946</v>
+        <v>-0.4569208076080828</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>53.35087572525482</v>
+        <v>53.35087570867936</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>18.71596748824224</v>
+        <v>18.71596746608034</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.6138150457568333</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-0.0331946142975589</v>
+        <v>-0.0331946142048453</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>50.53775997999208</v>
+        <v>50.53775997025562</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>14.15865910231082</v>
+        <v>14.15865905376505</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.7967174519968473</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-0.6491386695045893</v>
+        <v>-0.6491386691954912</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>43.12225406100386</v>
+        <v>43.12225418232757</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>22.38054407684219</v>
+        <v>22.38054412866609</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>1.18768695015543</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-0.1373228384012277</v>
+        <v>-0.1373228383600164</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>46.81840432107698</v>
+        <v>46.81840430210013</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>21.7707775535311</v>
+        <v>21.77077749463931</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.6583804777909603</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-0.6435658749770365</v>
+        <v>-0.643565874770982</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>31.40520725834228</v>
+        <v>31.40520728936709</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>31.76430029581225</v>
+        <v>31.76430034751797</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.5935163016092765</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-0.432055638247653</v>
+        <v>-0.432055638350679</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>52.36265183630773</v>
+        <v>52.36265181362887</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>11.76821157588596</v>
+        <v>11.76821147063815</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>1.226061382947103</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-0.7719051214151662</v>
+        <v>-0.7719051205909473</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>51.49284606380726</v>
+        <v>51.49284594553212</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>20.51854934176842</v>
+        <v>20.51854930293106</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.7428539184056693</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.6573987537099573</v>
+        <v>-0.6573987529887648</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>39.42266110270865</v>
+        <v>39.42266098019471</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>19.21547092785031</v>
+        <v>19.21547059189073</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.4466510469700749</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.202807712499418</v>
+        <v>-0.202807712458208</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>56.06641193645372</v>
+        <v>56.06641200533112</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>11.8522855934818</v>
+        <v>11.85228555976854</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>1.205540733118381</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.0244235282674772</v>
+        <v>0.0244235279583859</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>51.72157861351787</v>
+        <v>51.72157834613389</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>22.85334165184792</v>
+        <v>22.85334171903623</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.5696194355744605</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.09209491727709521</v>
+        <v>0.092094917751029</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>53.17181627950839</v>
+        <v>53.17181623945756</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>34.42896731883931</v>
+        <v>34.42896724117741</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.8248641393739227</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-0.4381415129767811</v>
+        <v>-0.4381415128531492</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>55.4349542641808</v>
+        <v>55.4349540793119</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>17.3148414656946</v>
+        <v>17.31484151680686</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.96071857287127</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.0676227412195461</v>
+        <v>0.06762274127105961</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>53.53780491331156</v>
+        <v>53.53780482616708</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>21.40331641367653</v>
+        <v>21.40331648554085</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.7700206972392768</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.2795373722086753</v>
+        <v>-0.2795373717965697</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>40.34834748546127</v>
+        <v>40.34834747845591</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>15.3849786805258</v>
+        <v>15.38497868418089</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.5750510777667147</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.6317816559670799</v>
+        <v>0.6317816559773695</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>51.8995597413733</v>
+        <v>51.89955968514139</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>12.07039592553</v>
+        <v>12.0703957768104</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.08527690054353371</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-0.0442507886772802</v>
+        <v>-0.044250788265172</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>432.9706652016063</v>
+        <v>432.9706652016062</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>51.7</v>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>50.96163231823188</v>
+        <v>50.96163202586099</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>6.549853241283897</v>
+        <v>6.549852891190266</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>1.735707428615535</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>1.098203139124188</v>
+        <v>1.09820315540277</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>53.90356627336945</v>
+        <v>53.90356625735447</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>8.86364285960617</v>
+        <v>8.863642832903487</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.7559556105341765</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>1.601730521423461</v>
+        <v>1.601730521938585</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4566,7 +4566,7 @@
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>428.1063434347074</v>
+        <v>428.1063434347072</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>31.45</v>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>50.12701565109003</v>
+        <v>50.12701530254636</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>23.507574736461</v>
+        <v>23.50757471890962</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.4721011747571447</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.2539445321693756</v>
+        <v>-0.2539445312421157</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>46.85334374115789</v>
+        <v>46.85334373203711</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>15.43148313784351</v>
+        <v>15.43148308491432</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.7612670615892232</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>13.45230301702439</v>
+        <v>13.45230301815764</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>61.90356580608247</v>
+        <v>61.90356562212491</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>15.95404141632878</v>
+        <v>15.95404140648106</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>1.473128958713068</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.175175311322133</v>
+        <v>0.1751753115900091</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>50.46443621497094</v>
+        <v>50.46443600362839</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>17.97892896414199</v>
+        <v>17.97892902301058</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.8449341680962054</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.0156707480318591</v>
+        <v>0.015670748103982</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>56.35866114372421</v>
+        <v>56.35866110094534</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>17.47595314318821</v>
+        <v>17.4759533055202</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0.7970022797668485</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.4590826113686887</v>
+        <v>0.4590826115953577</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>53.20537130084008</v>
+        <v>53.20537124568632</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>23.10145504292548</v>
+        <v>23.10145499839211</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.4512056850319863</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-1.057065988557143</v>
+        <v>-1.057065988371694</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>49.39499673394545</v>
+        <v>49.3949963759574</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>19.00354591378908</v>
+        <v>19.00354599185785</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>1.117857703745616</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.8945431894995755</v>
+        <v>-0.8945431873359684</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>50.85182085985326</v>
+        <v>50.85182080781991</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>30.95324210434352</v>
+        <v>30.95324219064291</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.6638388392793676</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-3.722637337258799</v>
+        <v>-3.722637336496365</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>47.63798667274189</v>
+        <v>47.63798665679957</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>17.34624390137674</v>
+        <v>17.34624385348305</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.4300690678661804</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-3.311493810537277</v>
+        <v>-3.311493810331221</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>39.86642228762798</v>
+        <v>39.86642195134134</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>19.0672912297797</v>
+        <v>19.06729136185881</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.8174207887863203</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.1135106719494787</v>
+        <v>0.1135106722585637</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5113,7 +5113,7 @@
         <v>51.04591535570363</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>10.74103951053982</v>
+        <v>10.74103951183171</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.7753672861968763</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.6174013104677091</v>
+        <v>-0.617401310673751</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>38.75331673513378</v>
+        <v>38.75331669662442</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>25.52088603280144</v>
+        <v>25.52088601883952</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.5776829284742635</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-2.529382724118776</v>
+        <v>-2.529382720409529</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>45.55050989186935</v>
+        <v>45.55050984048502</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>15.14421832456922</v>
+        <v>15.14421836164235</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.6157938542217407</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-0.8429556905178615</v>
+        <v>-0.8429556903324071</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>47.97880055018174</v>
+        <v>47.97880055425132</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>22.75822112188205</v>
+        <v>22.75822119311098</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>1.095275307900748</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>0.4140047813403482</v>
+        <v>0.4140047812373253</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>45.23602296111163</v>
+        <v>45.23602277372585</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>16.16673374689383</v>
+        <v>16.16673388552502</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.708523806779553</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-1.226681678897857</v>
+        <v>-1.226681676837298</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>347.3544989593393</v>
+        <v>347.3544989593394</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>4855</v>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>44.27907610302024</v>
+        <v>44.27907608531257</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>17.57909848661996</v>
+        <v>17.5790983642624</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>1.000054764253884</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-71.21050278739308</v>
+        <v>-71.21050278121098</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>38.92779103645388</v>
+        <v>38.92779101526649</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>26.89343176604868</v>
+        <v>26.893431730548</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.4181583126511264</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-1.657781831362216</v>
+        <v>-1.657781831259204</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>45.653214581001</v>
+        <v>45.65321453006408</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>24.38822368119112</v>
+        <v>24.38822351950636</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.683497449130963</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-1.714222822132113</v>
+        <v>-1.714222821101822</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5520,7 +5520,7 @@
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>333.6483663795637</v>
+        <v>333.6483663795635</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>1190</v>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>46.78307484757593</v>
+        <v>46.78307481712959</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>12.27985102358204</v>
+        <v>12.27985093765645</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.8258816358744208</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-1.82122917670403</v>
+        <v>-1.821229172170817</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>48.82298646959641</v>
+        <v>48.82298650456185</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>8.594937073077876</v>
+        <v>8.594937075064461</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.8488812645201096</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.1495561317572243</v>
+        <v>-0.1495561317366186</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5626,7 +5626,7 @@
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>327.3937655424172</v>
+        <v>327.3937655424171</v>
       </c>
       <c r="E98" s="2" t="n">
         <v>1820</v>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>48.60075316959789</v>
+        <v>48.60075315424942</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>14.21727160036192</v>
+        <v>14.2172715156228</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.5423860177252314</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-14.86631802799317</v>
+        <v>-14.86631802552048</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5679,7 +5679,7 @@
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>319.3103691554148</v>
+        <v>319.3103691554147</v>
       </c>
       <c r="E99" s="2" t="n">
         <v>93</v>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>42.4361154101081</v>
+        <v>42.43611537392408</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>15.88787810699281</v>
+        <v>15.88787796629373</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.5679184943403269</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.8437111640419568</v>
+        <v>-0.8437111637637873</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>51.76110131055167</v>
+        <v>51.76110118772823</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>26.33594710268452</v>
+        <v>26.33594720528338</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>1.47636021135205</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.0965042710631159</v>
+        <v>0.0965042716812948</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5785,7 +5785,7 @@
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>303.9868588376933</v>
+        <v>303.9868588376934</v>
       </c>
       <c r="E101" s="2" t="n">
         <v>26.45</v>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>44.49114844256012</v>
+        <v>44.49114841784677</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>21.60494770737755</v>
+        <v>21.60494774125333</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.5549106151562725</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>0.2905715284290453</v>
+        <v>0.290571528573285</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>35.20017672204797</v>
+        <v>35.20017626793532</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>33.85997596497661</v>
+        <v>33.85997599692163</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.5985921038756119</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>0.1869201647109042</v>
+        <v>0.1869201649993861</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>52.53229984503564</v>
+        <v>52.53229961296176</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>15.0148162845531</v>
+        <v>15.01481624793091</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.8751870139660766</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.0275949144513688</v>
+        <v>-0.027594914338032</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>42.68320431806602</v>
+        <v>42.68320404041521</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>20.82281505802341</v>
+        <v>20.82281513558968</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.6724974563376025</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>0.0909595527530988</v>
+        <v>0.090959553391879</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>41.89565912419543</v>
+        <v>41.89565906298297</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>24.96200531478559</v>
+        <v>24.96200548521961</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>0.3335130125837434</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>0.1805264993761333</v>
+        <v>0.1805264994791596</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>52.83216653464108</v>
+        <v>52.8321660848939</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>18.26901549301909</v>
+        <v>18.26901564042004</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.5635016753304125</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.1919878930734421</v>
+        <v>-0.1919878926716265</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6103,7 +6103,7 @@
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>261.2080428118373</v>
+        <v>261.2080428118372</v>
       </c>
       <c r="E107" s="2" t="n">
         <v>67</v>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>43.94801983306157</v>
+        <v>43.94801962543339</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>12.52934418206894</v>
+        <v>12.52934426412346</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.558585994699726</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.281472741290685</v>
+        <v>-0.2814727409609987</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>259.866964618029</v>
+        <v>259.8669646180288</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>17.4</v>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>45.38046543607606</v>
+        <v>45.38046515956176</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>16.77192277942702</v>
+        <v>16.77192277590919</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.9953561102034204</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.0077163296805471</v>
+        <v>-0.0077163293199449</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>48.2178090316519</v>
+        <v>48.21780904597536</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>15.61524664306522</v>
+        <v>15.61524665781917</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.2718052063818676</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.2509274731507775</v>
+        <v>0.2509274732950326</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>40.55806854105812</v>
+        <v>40.5580643523826</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>15.58868882261337</v>
+        <v>15.58868888188216</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.6625596030112977</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.1435709659848854</v>
+        <v>-0.1435709660260956</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>51.13745943910816</v>
+        <v>51.13745936286445</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>22.86870256218147</v>
+        <v>22.86870251618441</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.7769152664504929</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.0673648945762928</v>
+        <v>0.06736489443204489</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>241.7473673291414</v>
+        <v>241.7473673291413</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>40.15</v>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>49.29943889820353</v>
+        <v>49.29943987337887</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>16.73167871043117</v>
+        <v>16.73167868145203</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.9929101742909836</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.1509990190611388</v>
+        <v>0.1509990190817389</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>46.35527653268856</v>
+        <v>46.35527646348658</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>20.81729326051425</v>
+        <v>20.81729331281481</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.6843485682622978</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.1124581835510283</v>
+        <v>-0.112458183334663</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>42.37569307657395</v>
+        <v>42.37569299609675</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>25.42553025086282</v>
+        <v>25.42553020469853</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>1.189051952011658</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-3.507820634904373</v>
+        <v>-3.507820632019602</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6541,7 +6541,7 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>5.894406618521231</v>
+        <v>5.894406613722722</v>
       </c>
       <c r="I115" s="2" t="n">
         <v>16.71609921062464</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-7.883995480695214</v>
+        <v>-7.883995480592174</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>39.75755771223096</v>
+        <v>39.75755769374807</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>30.83862751792328</v>
+        <v>30.83862755179342</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.6698314200703324</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>0.2762207405965009</v>
+        <v>0.276220740720136</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>42.96876277706797</v>
+        <v>42.96876276109524</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>12.63026796776372</v>
+        <v>12.63026809592015</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>1.127752941825462</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.2348524876921436</v>
+        <v>-0.2348524876097205</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6703,7 +6703,7 @@
         <v>46.22371657196188</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>13.09985948092228</v>
+        <v>13.09985949960422</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.6016487148817888</v>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>50.70272087333871</v>
+        <v>50.7027208782856</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>12.23041601909402</v>
+        <v>12.23041601758287</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>0.1557842148340412</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.1616634286105926</v>
+        <v>-0.1616634287136236</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>31.03862485121311</v>
+        <v>31.03862456624346</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>15.60763883856227</v>
+        <v>15.60763886728877</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>0.6842935196071651</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.63464798829632</v>
+        <v>-0.6346479878429827</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>44.1878915404678</v>
+        <v>44.18789155363981</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>15.98242005140424</v>
+        <v>15.98242006336745</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.7151020875209576</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>0.0912139576670255</v>
+        <v>0.09121395768762711</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>43.84307104766052</v>
+        <v>43.84307068692377</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>15.54868382726068</v>
+        <v>15.54868414351743</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>0.8135508499803757</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-1.948465043567257</v>
+        <v>-1.94846503944606</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>44.66954226179125</v>
+        <v>44.66954198617165</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>13.48537739176632</v>
+        <v>13.4853774863357</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>0.1426456941433795</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.0930713919733152</v>
+        <v>-0.09307139162301691</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7004,7 +7004,7 @@
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>110.6312253399946</v>
+        <v>110.6312253399937</v>
       </c>
       <c r="E124" s="2" t="n">
         <v>24.3</v>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>32.96035509944109</v>
+        <v>32.96035511874453</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>10.22277766602677</v>
+        <v>10.22277769491396</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>1.012130694739113</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>0.0227745384791415</v>
+        <v>0.0227745384276294</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7057,7 +7057,7 @@
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>102.6341827157463</v>
+        <v>102.6341827157464</v>
       </c>
       <c r="E125" s="2" t="n">
         <v>25</v>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>26.3168876974246</v>
+        <v>26.31688764267237</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>17.98143418133377</v>
+        <v>17.98143414005698</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>1.090408660595745</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>0.0104356081022597</v>
+        <v>0.0104356081331671</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>

</xml_diff>